<commit_message>
feat(analysis): add individual XLSX downloads and refine button layout
Provide separate claim, channel, and type workbooks with matching hashes and generation checks. Place downloads in section action areas with a separate mobile row, and style the JSON download as a right-aligned button.
</commit_message>
<xml_diff>
--- a/assets/analysis/analysis_data.xlsx
+++ b/assets/analysis/analysis_data.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주장 309건" sheetId="1" r:id="Re36b927d66e94957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="채널별 집계" sheetId="2" r:id="R26b3ff40a3eb43fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="유형별 집계" sheetId="3" r:id="R8771bd6cae5f4b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주장 309건" sheetId="1" r:id="R33a470acd31b404f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="채널별 집계" sheetId="2" r:id="R335062a52bf64e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="유형별 집계" sheetId="3" r:id="R8119d093597a4e03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20615,7 +20615,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R315f17c3e4174a3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R035957058f314d89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21958,7 +21958,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ea16d1beb024b16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc238f714963042a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22245,7 +22245,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8e3c860302544e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1485308e34c149d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>